<commit_message>
Add UK eyelash serum feed, stock 2, refresh price table
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTewxUJQKBNDwnYyc7b6kM
</commit_message>
<xml_diff>
--- a/Prices_UK_DE_2026-10-26.xlsx
+++ b/Prices_UK_DE_2026-10-26.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,7 +514,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>В фиде</t>
+          <t>Остаток</t>
         </is>
       </c>
     </row>
@@ -526,45 +526,45 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4751045860468</t>
+          <t>4751045863438</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Масло для ногтей</t>
+          <t>Шампунь ладан</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4751045860468_mfn</t>
+          <t>4751045863438_mfn</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6.55</v>
+        <v>19.72</v>
       </c>
       <c r="F2" t="n">
-        <v>5.5</v>
+        <v>16.56</v>
       </c>
       <c r="G2" t="n">
-        <v>7.15</v>
+        <v>21.53</v>
       </c>
       <c r="H2" t="n">
-        <v>7.94</v>
+        <v>23.92</v>
       </c>
       <c r="J2" t="n">
-        <v>7.15</v>
+        <v>21.53</v>
       </c>
       <c r="K2" t="n">
-        <v>6.6</v>
+        <v>19.88</v>
       </c>
       <c r="L2" t="n">
-        <v>9.529999999999999</v>
+        <v>28.7</v>
       </c>
       <c r="M2" t="n">
-        <v>6.94</v>
+        <v>20.88</v>
       </c>
       <c r="N2" t="n">
-        <v>6.65</v>
+        <v>20.02</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -581,16 +581,14 @@
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Sale, Your, List, Min, Max; Business и цены от шт. в шаблонах нет</t>
-        </is>
+      <c r="R2" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -612,31 +610,28 @@
         <v>19.72</v>
       </c>
       <c r="F3" t="n">
-        <v>19.72</v>
+        <v>16.56</v>
       </c>
       <c r="G3" t="n">
-        <v>25.64</v>
+        <v>21.53</v>
       </c>
       <c r="H3" t="n">
-        <v>28.49</v>
-      </c>
-      <c r="I3" t="n">
-        <v>23.94</v>
+        <v>23.92</v>
       </c>
       <c r="J3" t="n">
-        <v>25.64</v>
+        <v>21.53</v>
       </c>
       <c r="K3" t="n">
-        <v>23.66</v>
+        <v>19.88</v>
       </c>
       <c r="L3" t="n">
-        <v>34.19</v>
+        <v>28.7</v>
       </c>
       <c r="M3" t="n">
-        <v>24.87</v>
+        <v>20.88</v>
       </c>
       <c r="N3" t="n">
-        <v>23.85</v>
+        <v>20.02</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -653,62 +648,57 @@
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Sale, Your, List, UVP, Min, Max; Business и цены от шт. в шаблонах нет</t>
-        </is>
+      <c r="R3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4751045863360</t>
+          <t>4751045863421</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Кондиционер арган</t>
+          <t>Шампунь арган</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4751045863360_mfn</t>
+          <t>4751045863421_mfn</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>6.26</v>
       </c>
       <c r="F4" t="n">
-        <v>6.26</v>
+        <v>5.26</v>
       </c>
       <c r="G4" t="n">
-        <v>8.140000000000001</v>
+        <v>6.84</v>
       </c>
       <c r="H4" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="I4" t="n">
         <v>7.6</v>
       </c>
       <c r="J4" t="n">
-        <v>8.140000000000001</v>
+        <v>6.84</v>
       </c>
       <c r="K4" t="n">
-        <v>7.51</v>
+        <v>6.31</v>
       </c>
       <c r="L4" t="n">
-        <v>10.85</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="M4" t="n">
-        <v>7.9</v>
+        <v>6.63</v>
       </c>
       <c r="N4" t="n">
-        <v>7.57</v>
+        <v>6.36</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -725,62 +715,57 @@
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Sale, Your, List, UVP, Min, Max; Business и цены от шт. в шаблонах нет</t>
-        </is>
+      <c r="R4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4751045860468</t>
+          <t>4751045863360</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Масло для ногтей</t>
+          <t>Кондиционер арган</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4751045860468_mfn</t>
+          <t>4751045863360_mfn</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>6.55</v>
+        <v>6.26</v>
       </c>
       <c r="F5" t="n">
-        <v>6.55</v>
+        <v>5.26</v>
       </c>
       <c r="G5" t="n">
-        <v>8.52</v>
+        <v>6.84</v>
       </c>
       <c r="H5" t="n">
-        <v>9.470000000000001</v>
-      </c>
-      <c r="I5" t="n">
-        <v>7.96</v>
+        <v>7.6</v>
       </c>
       <c r="J5" t="n">
-        <v>8.52</v>
+        <v>6.84</v>
       </c>
       <c r="K5" t="n">
-        <v>7.86</v>
+        <v>6.31</v>
       </c>
       <c r="L5" t="n">
-        <v>11.36</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>8.26</v>
+        <v>6.63</v>
       </c>
       <c r="N5" t="n">
-        <v>7.92</v>
+        <v>6.36</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -797,82 +782,973 @@
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Sale, Your, List, UVP, Min, Max; Business и цены от шт. в шаблонах нет</t>
-        </is>
+      <c r="R5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4751045860024</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Бальзам ши/мирра/ладан</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4751045860024_mfn</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="G6" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="J6" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="K6" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="L6" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="N6" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4751045860314</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Бальзам для глаз</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4751045860314_mfn</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4751045860451</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Сыворотка лаванда</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4751045860451_mfn</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4751045860468</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Масло для ногтей</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4751045860468_mfn</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="J9" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="K9" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="L9" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="M9" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="N9" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4751045863438</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Шампунь ладан</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4751045863438_mfn</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="F10" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="G10" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="H10" t="n">
+        <v>28.49</v>
+      </c>
+      <c r="I10" t="n">
+        <v>23.94</v>
+      </c>
+      <c r="J10" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="K10" t="n">
+        <v>23.66</v>
+      </c>
+      <c r="L10" t="n">
+        <v>34.19</v>
+      </c>
+      <c r="M10" t="n">
+        <v>24.87</v>
+      </c>
+      <c r="N10" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>4751045863421</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Шампунь арган</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>4751045863421_mfn</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="G11" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="I11" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="K11" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="L11" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="M11" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="N11" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4751045860024</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Бальзам ши/мирра/ладан</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>4751045860024_mfn</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H12" t="n">
+        <v>13</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="J12" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="M12" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="N12" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4751045860314</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Бальзам для глаз</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4751045860314_mfn</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="L13" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="M13" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4751045860451</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Сыворотка лаванда</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4751045860451_mfn</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="M14" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4751045863490</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Кондиционер ладан</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4751045863490_mfn</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="F15" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="G15" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="H15" t="n">
+        <v>28.49</v>
+      </c>
+      <c r="I15" t="n">
+        <v>23.94</v>
+      </c>
+      <c r="J15" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="K15" t="n">
+        <v>23.66</v>
+      </c>
+      <c r="L15" t="n">
+        <v>34.19</v>
+      </c>
+      <c r="M15" t="n">
+        <v>24.87</v>
+      </c>
+      <c r="N15" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>4751045863360</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Кондиционер арган</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>4751045863360_mfn</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="G16" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="H16" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="J16" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="K16" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="L16" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="M16" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="N16" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>4751045860468</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Масло для ногтей</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4751045860468_mfn</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="G17" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="H17" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="I17" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="K17" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="L17" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M17" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="N17" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>4751045860437</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Сыворотка ресницы</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>4751045860437_mfn</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E18" t="n">
         <v>6.78</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F18" t="n">
         <v>6.78</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G18" t="n">
         <v>8.81</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H18" t="n">
         <v>9.789999999999999</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I18" t="n">
         <v>8.23</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J18" t="n">
         <v>8.81</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K18" t="n">
         <v>8.140000000000001</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L18" t="n">
         <v>11.75</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M18" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N18" t="n">
         <v>8.19</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>2027-05-01</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Sale, Your, List, UVP, Min, Max; Business и цены от шт. в шаблонах нет</t>
-        </is>
+      <c r="R18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>4751045860437</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Сыворотка ресницы</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>4751045860437_mfn</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G19" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="J19" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="K19" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="L19" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="M19" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="N19" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -886,34 +1762,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>UK: H×0.84 (1 EUR = 0.84 GBP), затем ×1.30. DE: EUR без пересчёта.</t>
+          <t>UK: H×0.84, затем ×1.30. DE: EUR.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Business и цены от 2/4 шт. в шаблонах отсутствуют, в фид не записаны. Проценты 3% и 7% — моё предложение: цена от 4 шт. не ниже Min (H×1.20).</t>
+          <t>Business Price и цены от 2/4 шт. посчитаны, но в фиды НЕ записаны: в скачанных шаблонах нет группы Offer (Amazon Business). Проценты 3% и 7% — предложение.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UVP в DE-шаблоне указывается без налога: Your Price / 1.19 (НДС 19%, допущение).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Quantity (остаток) в фидах = 0, пока не дадите количество.</t>
+          <t>UVP в DE без налога: Your/1.19 (допущение).</t>
         </is>
       </c>
     </row>

</xml_diff>